<commit_message>
Actualización: Plantillas y archivos de ayer
</commit_message>
<xml_diff>
--- a/plantillas/plantillla_creacion_temas_usuarios_owners.xlsx
+++ b/plantillas/plantillla_creacion_temas_usuarios_owners.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_Aprovicionamiento_M365\archivos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_Aprovicionamiento_M365\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8D125F2-DD11-4FC8-91BD-3378681DD297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCC61E2-61C3-4F53-ABF7-0B04293AA933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Grado</t>
   </si>
@@ -64,21 +64,6 @@
   </si>
   <si>
     <t>NOVENO</t>
-  </si>
-  <si>
-    <t>MATEMÁTICAS</t>
-  </si>
-  <si>
-    <t>ddiaz@calasanzsuba.edu.co</t>
-  </si>
-  <si>
-    <t>jsanchez@calasanzsuba.edu.co</t>
-  </si>
-  <si>
-    <t>lhenao@calasanzsuba.edu.co</t>
-  </si>
-  <si>
-    <t>solaya@calasanzsuba.edu.co</t>
   </si>
 </sst>
 </file>
@@ -508,40 +493,19 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2">
-        <v>901</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="3"/>
       <c r="E2" s="2" t="str">
         <f>B2 &amp; ": "&amp; C2</f>
-        <v>901: MATEMÁTICAS</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>14</v>
-      </c>
+        <v xml:space="preserve">: </v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{744591B4-AB7A-425B-8130-C9FF08173FEA}"/>
-    <hyperlink ref="G2" r:id="rId2" xr:uid="{FC503A70-D6E2-4A7A-B20F-83722DCDB976}"/>
-    <hyperlink ref="H2" r:id="rId3" xr:uid="{F8F94FE0-2304-4DAA-A9D7-FB36D37FEC32}"/>
-    <hyperlink ref="I2" r:id="rId4" xr:uid="{D89AC7C4-8C66-40C7-969B-F6B17A64FA08}"/>
-    <hyperlink ref="D2" r:id="rId5" xr:uid="{4EA479BE-D273-457C-B62A-60545C7EC82C}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>